<commit_message>
Split into frontend/backend, add backend scaffold, refresh vendor thread charts
- Move the Vite React app into frontend/ and add a new backend/ FastAPI
  service scaffold (domain models, migrations, workbook profiling tools)
  for the eventual move off the local mock data layer.
- Regenerate frontend/public/data/color-mappings.json from the latest
  Thread Chart vendor workbooks, including several newly added vendors.
- Fix the Finder page's thread combobox rendering behind the match card
  (stacking-context fix on .finder-controls) and relabel the PMS swatch
  as "Monitor Display Color" to match the source spreadsheet terminology.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Thread Chart/AP Specialties Thread Charts.xlsx
+++ b/Thread Chart/AP Specialties Thread Charts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\fs1\InformationManagement\Procedures &amp; References\Embroidery Thread Charts\Completed\AP Specialties\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12FD2EE-3766-4F07-B22C-1DEB55B9874C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{38EDBD1E-D69D-4B50-8AF7-3BFDBAF90187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22920" yWindow="-1095" windowWidth="29040" windowHeight="15840" xr2:uid="{F028543A-CA1A-4C22-838B-894A262A5CAB}"/>
+    <workbookView xWindow="19090" yWindow="-5720" windowWidth="38620" windowHeight="21100" xr2:uid="{F028543A-CA1A-4C22-838B-894A262A5CAB}"/>
   </bookViews>
   <sheets>
     <sheet name="RA Super Strength Rayon" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RA Super Strength Rayon'!$A$1:$I$15</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +26,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -48,6 +53,9 @@
     <t>Thread Number</t>
   </si>
   <si>
+    <t>Monitor Display Color</t>
+  </si>
+  <si>
     <t>PMS Number</t>
   </si>
   <si>
@@ -60,88 +68,85 @@
     <t>B</t>
   </si>
   <si>
+    <t>Black</t>
+  </si>
+  <si>
+    <t>Blacks</t>
+  </si>
+  <si>
     <t>RA SSR 9</t>
   </si>
   <si>
+    <t>BlackC</t>
+  </si>
+  <si>
+    <t>Pacific Blue</t>
+  </si>
+  <si>
+    <t>Blues</t>
+  </si>
+  <si>
+    <t>Sapphire</t>
+  </si>
+  <si>
+    <t>Light Navy</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>Browns</t>
+  </si>
+  <si>
+    <t>Banner Gray</t>
+  </si>
+  <si>
+    <t>Grays</t>
+  </si>
+  <si>
+    <t>Kelly</t>
+  </si>
+  <si>
+    <t>Greens</t>
+  </si>
+  <si>
+    <t>Evergreen</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Oranges</t>
+  </si>
+  <si>
+    <t>Purple Shadow</t>
+  </si>
+  <si>
+    <t>Purples</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>Reds</t>
+  </si>
+  <si>
+    <t>Burgundy</t>
+  </si>
+  <si>
+    <t>Snow White</t>
+  </si>
+  <si>
+    <t>Whites</t>
+  </si>
+  <si>
+    <t>Trans. White</t>
+  </si>
+  <si>
     <t>Goldenrod</t>
   </si>
   <si>
-    <t>Grays</t>
-  </si>
-  <si>
-    <t>Banner Gray</t>
-  </si>
-  <si>
-    <t>Orange</t>
-  </si>
-  <si>
-    <t>Sapphire</t>
-  </si>
-  <si>
-    <t>Light Navy</t>
-  </si>
-  <si>
-    <t>Pacific Blue</t>
-  </si>
-  <si>
-    <t>Red</t>
-  </si>
-  <si>
-    <t>Burgundy</t>
-  </si>
-  <si>
-    <t>Purple Shadow</t>
-  </si>
-  <si>
-    <t>Greens</t>
-  </si>
-  <si>
-    <t>Purples</t>
-  </si>
-  <si>
-    <t>Reds</t>
-  </si>
-  <si>
-    <t>Blues</t>
-  </si>
-  <si>
-    <t>Oranges</t>
-  </si>
-  <si>
     <t>Yellows</t>
-  </si>
-  <si>
-    <t>Kelly</t>
-  </si>
-  <si>
-    <t>Evergreen</t>
-  </si>
-  <si>
-    <t>Browns</t>
-  </si>
-  <si>
-    <t>Brown</t>
-  </si>
-  <si>
-    <t>Monitor Display Color</t>
-  </si>
-  <si>
-    <t>Black</t>
-  </si>
-  <si>
-    <t>Blacks</t>
-  </si>
-  <si>
-    <t>BlackC</t>
-  </si>
-  <si>
-    <t>Snow White</t>
-  </si>
-  <si>
-    <t>Whites</t>
-  </si>
-  <si>
-    <t>Trans. White</t>
   </si>
 </sst>
 </file>
@@ -151,7 +156,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -671,8 +676,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A968E8BA-6A80-456B-8B85-E8C99657187B}">
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O18"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col min="1" max="1" width="20.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.7109375" style="1" customWidth="1"/>
@@ -680,14 +685,14 @@
     <col min="4" max="4" width="19.7109375" style="18" customWidth="1"/>
     <col min="5" max="5" width="50.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="17.7109375" style="1" customWidth="1"/>
-    <col min="7" max="9" width="8.85546875" style="1"/>
-    <col min="10" max="10" width="20.7109375" style="1" customWidth="1"/>
-    <col min="11" max="14" width="8.85546875" style="1"/>
-    <col min="15" max="15" width="50.7109375" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.85546875" style="1"/>
+    <col min="7" max="9" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" style="1" hidden="1" customWidth="1"/>
+    <col min="11" max="14" width="8.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="50.7109375" style="1" hidden="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.85546875" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="50.1" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -701,37 +706,37 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="50.1" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D2" s="18">
         <v>2296</v>
       </c>
       <c r="E2" s="15"/>
       <c r="F2" s="1" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="G2" s="1">
         <v>0</v>
@@ -743,15 +748,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="50.1" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D3" s="18">
         <v>2388</v>
@@ -770,15 +775,15 @@
         <v>185</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="50.1" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D4" s="18">
         <v>2280</v>
@@ -797,15 +802,15 @@
         <v>185</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="50.1" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D5" s="18">
         <v>2303</v>
@@ -824,15 +829,15 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="50.1" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D6" s="18">
         <v>2251</v>
@@ -851,15 +856,15 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="50.1" customHeight="1">
       <c r="A7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="D7" s="18">
         <v>2585</v>
@@ -878,15 +883,15 @@
         <v>172</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="50.1" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D8" s="18">
         <v>2240</v>
@@ -905,15 +910,15 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="50.1" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D9" s="18">
         <v>2315</v>
@@ -932,15 +937,15 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="50.1" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D10" s="18">
         <v>2218</v>
@@ -959,15 +964,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="50.1" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D11" s="19">
         <v>2430</v>
@@ -986,15 +991,15 @@
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="50.1" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D12" s="19">
         <v>2378</v>
@@ -1013,15 +1018,15 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="50.1" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D13" s="19">
         <v>2249</v>
@@ -1040,22 +1045,22 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="50.1" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D14" s="19">
         <v>2297</v>
       </c>
       <c r="E14" s="16"/>
       <c r="F14" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G14" s="1">
         <v>255</v>
@@ -1067,15 +1072,15 @@
         <v>255</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="50.1" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D15" s="19">
         <v>2242</v>
@@ -1094,11 +1099,11 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="50.1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:9" ht="50.1" hidden="1" customHeight="1"/>
+    <row r="17" ht="50.1" hidden="1" customHeight="1"/>
+    <row r="18" ht="50.1" hidden="1" customHeight="1"/>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="vhwREJ5baEUNyXlA2Mg5KcyIfiRETM1s4XdsCc9hSQoeONG9+IkpP4Z9SZril8YhNZK77PDAb3BwQ4exxafRSQ==" saltValue="aAuka+ZthmwjQvQsXT/2pA==" spinCount="100000" sheet="1" objects="1" scenarios="1" sort="0" autoFilter="0"/>
+  <sheetProtection sort="0" autoFilter="0"/>
   <protectedRanges>
     <protectedRange sqref="A1:I15" name="AllowSortFilter"/>
   </protectedRanges>
@@ -1109,4 +1114,225 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ea7a09a4-fe73-437e-8a86-996460e9b058">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a2b9d960-66d6-4e1d-a64a-950bc94b8bb0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A1C7DD37AE641E4B9B3FD2F75B2D99BC" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6b9cb41f595aff4764e09aef2b23c1ed">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ea7a09a4-fe73-437e-8a86-996460e9b058" xmlns:ns3="a2b9d960-66d6-4e1d-a64a-950bc94b8bb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="daad8a4a6daff5298e6b89d91afce8e3" ns2:_="" ns3:_="">
+    <xsd:import namespace="ea7a09a4-fe73-437e-8a86-996460e9b058"/>
+    <xsd:import namespace="a2b9d960-66d6-4e1d-a64a-950bc94b8bb0"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea7a09a4-fe73-437e-8a86-996460e9b058" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="d2f5926c-fefe-46c4-85d9-9ef0eea46f5c" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a2b9d960-66d6-4e1d-a64a-950bc94b8bb0" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{6fbb2a74-2168-4404-a595-59f9a11d4eed}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="a2b9d960-66d6-4e1d-a64a-950bc94b8bb0">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{802E0836-D821-4DB9-A847-E2ABC0101918}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF28046F-FC63-490E-8823-D1C8B4080E74}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79040919-24BF-47B3-8455-B4C8CB480836}"/>
 </file>
</xml_diff>